<commit_message>
Kit gratis (Excel): actualizar logo viejo -> nuevo isotipo MM Menttor en las 8 hojas
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/landing/assets/Menttor_Kit_Inicio_Rapido.xlsx
+++ b/landing/assets/Menttor_Kit_Inicio_Rapido.xlsx
@@ -1,498 +1,33 @@
 
-<file path=docProps\app.xml><?xml version="1.0" encoding="utf-8"?>
-<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <Application>Microsoft Excel</Application>
-  <DocSecurity>0</DocSecurity>
-  <ScaleCrop>false</ScaleCrop>
-  <HeadingPairs>
-    <vt:vector size="2" baseType="variant">
-      <vt:variant>
-        <vt:lpstr>Hojas de cálculo</vt:lpstr>
-      </vt:variant>
-      <vt:variant>
-        <vt:i4>9</vt:i4>
-      </vt:variant>
-    </vt:vector>
-  </HeadingPairs>
-  <TitlesOfParts>
-    <vt:vector size="9" baseType="lpstr">
-      <vt:lpstr>Instrucciones</vt:lpstr>
-      <vt:lpstr>Charter 1-Pager</vt:lpstr>
-      <vt:lpstr>Checklist Kickoff</vt:lpstr>
-      <vt:lpstr>Lista</vt:lpstr>
-      <vt:lpstr>RACI (Plantilla)</vt:lpstr>
-      <vt:lpstr>RACI (Ejemplo)</vt:lpstr>
-      <vt:lpstr>Minuta Ejecutiva</vt:lpstr>
-      <vt:lpstr>Roadmap 8 Semanas</vt:lpstr>
-      <vt:lpstr>Definiciones</vt:lpstr>
-    </vt:vector>
-  </TitlesOfParts>
-  <Company/>
-  <LinksUpToDate>false</LinksUpToDate>
-  <SharedDoc>false</SharedDoc>
-  <HyperlinksChanged>false</HyperlinksChanged>
-  <AppVersion>16.0300</AppVersion>
-</Properties>
+<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30228"/>
+  <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JOSEMO~1\AppData\Local\Temp\claude\C--Users-Jose-Montilla-OneDrive-Cloude-pagina-web-MM\82739746-f994-4b96-ab4e-13fcee2a012b\scratchpad\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA0460D5-B49B-4573-8F08-5C555BB9227C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="808" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
+  <sheets>
+    <sheet name="Instrucciones" sheetId="1" r:id="rId1"/>
+    <sheet name="Charter 1-Pager" sheetId="3" r:id="rId2"/>
+    <sheet name="Checklist Kickoff" sheetId="2" r:id="rId3"/>
+    <sheet name="Lista" sheetId="8" state="hidden" r:id="rId4"/>
+    <sheet name="RACI (Plantilla)" sheetId="4" r:id="rId5"/>
+    <sheet name="RACI (Ejemplo)" sheetId="5" r:id="rId6"/>
+    <sheet name="Minuta Ejecutiva" sheetId="6" r:id="rId7"/>
+    <sheet name="Roadmap 8 Semanas" sheetId="7" r:id="rId8"/>
+    <sheet name="Definiciones" sheetId="9" r:id="rId9"/>
+  </sheets>
+  <calcPr calcId="124519"/>
+</workbook>
 </file>
 
-<file path=docProps\core.xml><?xml version="1.0" encoding="utf-8"?>
-<cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:dcmitype="http://purl.org/dc/dcmitype/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
-  <dc:creator>clara.magin@cermaq.com</dc:creator>
-  <cp:lastModifiedBy>Clara Magin</cp:lastModifiedBy>
-  <dcterms:created xsi:type="dcterms:W3CDTF">2025-10-31T19:18:40Z</dcterms:created>
-  <dcterms:modified xsi:type="dcterms:W3CDTF">2025-11-07T12:08:53Z</dcterms:modified>
-</cp:coreProperties>
-</file>
-
-<file path=xl\drawings\drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>2072640</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>86052</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Imagen 2">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{67D72CB7-AAAB-917C-D8A3-E07AC81F72E9}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill rotWithShape="1">
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect l="8051" t="15466" r="8051" b="15042"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="2072640" cy="1716732"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl\drawings\drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>2072640</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>177492</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Imagen 2">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{963365F3-ECA3-4BFD-917E-55B01BE4235D}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill rotWithShape="1">
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect l="8051" t="15466" r="8051" b="15042"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="2072640" cy="1716732"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl\drawings\drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>2072640</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>131772</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Imagen 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{675F9C0C-0CD7-4808-AE64-EE81734517CA}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill rotWithShape="1">
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect l="8051" t="15466" r="8051" b="15042"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="2072640" cy="1716732"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl\drawings\drawing4.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>2072640</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>160559</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Imagen 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5CF84C2F-16CE-4D8D-B594-235D2C44120D}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill rotWithShape="1">
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect l="8051" t="15466" r="8051" b="15042"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="2072640" cy="1715039"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl\drawings\drawing5.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>2072640</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>130079</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Imagen 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{29BDEBA4-B0C5-4DFE-B119-51BD15BFE596}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill rotWithShape="1">
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect l="8051" t="15466" r="8051" b="15042"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="2072640" cy="1715039"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl\drawings\drawing6.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>130079</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Imagen 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2606413F-30AB-41A1-8289-A17C247EB2DA}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill rotWithShape="1">
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect l="8051" t="15466" r="8051" b="15042"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="2072640" cy="1715039"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl\drawings\drawing7.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>2072640</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>160559</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Imagen 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{60690204-2552-495C-89A1-448892BF5AC7}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill rotWithShape="1">
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect l="8051" t="15466" r="8051" b="15042"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="2072640" cy="1715039"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl\drawings\drawing8.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>2072640</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>177492</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Imagen 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BC752C58-BB8F-4E58-BD09-5A9D68679548}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill rotWithShape="1">
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect l="8051" t="15466" r="8051" b="15042"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="2072640" cy="1716732"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl\sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="128">
   <si>
     <t>Bienvenida/o al Kit de Inicio Rápido – Menttor</t>
@@ -881,7 +416,7 @@
 </sst>
 </file>
 
-<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="5" x14ac:knownFonts="1">
     <font>
@@ -1041,7 +576,447 @@
 </styleSheet>
 </file>
 
-<file path=xl\theme\theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>2072640</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>222780</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Imagen 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0B36EA55-F646-850D-D599-6A52FEAFD52E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="2072640" cy="651405"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>2072640</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>222780</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Imagen 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4DD91091-5757-10EC-41C5-7BA5669C8B17}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="2072640" cy="651405"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>2034540</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>184347</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Imagen 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DCA4B3D6-AC33-723C-98FD-1B6D3CFBFFD3}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="2034540" cy="639430"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>2063115</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>219786</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Imagen 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D33DA621-7111-13D5-1368-73C2C1845BCE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="2063115" cy="648411"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>2015490</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>185768</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Imagen 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D82E59FB-E6BF-351D-6AC3-2AED3B60777B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="2015490" cy="633443"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>186966</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Imagen 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9374BFF1-C3BC-5BF8-E72D-65C556BF927B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="2019300" cy="634641"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>2034540</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>210805</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Imagen 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6BF38672-04AB-2C08-71B1-2694968A08E1}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="2034540" cy="639430"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing8.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>2072640</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>222780</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Imagen 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F730F1E2-3DF5-7BE4-CE4A-E67123706F00}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="2072640" cy="651405"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
     <a:clrScheme name="Office 2007 - 2010">
@@ -1326,109 +1301,81 @@
 </a:theme>
 </file>
 
-<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29127"/>
-  <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\internal1.com\cermaq-cl\Home1-PMO\clmag\CachedDoc\My Documents\MM Mentor\Kits\DOC GRATIS\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{25DDA6E6-7BC8-4150-BD84-4F2B98BEFE50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="808" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-  </bookViews>
-  <sheets>
-    <sheet name="Instrucciones" sheetId="1" r:id="rId1"/>
-    <sheet name="Charter 1-Pager" sheetId="3" r:id="rId2"/>
-    <sheet name="Checklist Kickoff" sheetId="2" r:id="rId3"/>
-    <sheet name="Lista" sheetId="8" state="hidden" r:id="rId4"/>
-    <sheet name="RACI (Plantilla)" sheetId="4" r:id="rId5"/>
-    <sheet name="RACI (Ejemplo)" sheetId="5" r:id="rId6"/>
-    <sheet name="Minuta Ejecutiva" sheetId="6" r:id="rId7"/>
-    <sheet name="Roadmap 8 Semanas" sheetId="7" r:id="rId8"/>
-    <sheet name="Definiciones" sheetId="9" r:id="rId9"/>
-  </sheets>
-  <calcPr calcId="124519"/>
-</workbook>
-</file>
-
-<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B2:B17"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="33" customWidth="1"/>
-    <col min="2" max="2" width="96.88671875" customWidth="1"/>
+    <col min="2" max="2" width="96.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:2" ht="18" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:2" ht="18.75" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="3" spans="2:2" ht="19.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:2" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="2"/>
     </row>
-    <row r="4" spans="2:2" ht="19.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:2" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="2:2" ht="19.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:2" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="2"/>
     </row>
-    <row r="6" spans="2:2" ht="19.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:2" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="2:2" ht="19.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:2" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="2:2" ht="19.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:2" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="2" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="9" spans="2:2" ht="19.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:2" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="10" spans="2:2" ht="19.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:2" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="2:2" ht="19.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:2" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="2:2" ht="19.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:2" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="2" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="13" spans="2:2" ht="19.2" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="14" spans="2:2" ht="18" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:2" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="14" spans="2:2" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B14" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="15" spans="2:2" ht="18" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:2" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B15" s="2"/>
     </row>
-    <row r="16" spans="2:2" ht="25.2" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="2:2" ht="25.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B16" s="3" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="17" spans="2:2" ht="21" x14ac:dyDescent="0.4">
+    <row r="17" spans="2:2" ht="21" x14ac:dyDescent="0.35">
       <c r="B17" s="3" t="s">
         <v>106</v>
       </c>
@@ -1439,16 +1386,16 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="B2:C16"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="34.5546875" customWidth="1"/>
-    <col min="2" max="3" width="43.44140625" customWidth="1"/>
+    <col min="1" max="1" width="34.5703125" customWidth="1"/>
+    <col min="2" max="3" width="43.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:3" ht="18" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:3" ht="18.75" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
         <v>82</v>
       </c>
@@ -1456,85 +1403,85 @@
         <v>83</v>
       </c>
     </row>
-    <row r="3" spans="2:3" ht="22.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:3" ht="22.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="4" t="s">
         <v>104</v>
       </c>
       <c r="C3" s="5"/>
     </row>
-    <row r="4" spans="2:3" ht="22.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:3" ht="22.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="4" t="s">
         <v>29</v>
       </c>
       <c r="C4" s="5"/>
     </row>
-    <row r="5" spans="2:3" ht="22.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:3" ht="22.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="4" t="s">
         <v>30</v>
       </c>
       <c r="C5" s="5"/>
     </row>
-    <row r="6" spans="2:3" ht="22.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:3" ht="22.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="4" t="s">
         <v>31</v>
       </c>
       <c r="C6" s="5"/>
     </row>
-    <row r="7" spans="2:3" ht="22.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:3" ht="22.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="4" t="s">
         <v>32</v>
       </c>
       <c r="C7" s="5"/>
     </row>
-    <row r="8" spans="2:3" ht="22.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:3" ht="22.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="4" t="s">
         <v>33</v>
       </c>
       <c r="C8" s="5"/>
     </row>
-    <row r="9" spans="2:3" ht="22.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:3" ht="22.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="4" t="s">
         <v>34</v>
       </c>
       <c r="C9" s="5"/>
     </row>
-    <row r="10" spans="2:3" ht="22.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:3" ht="22.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="4" t="s">
         <v>35</v>
       </c>
       <c r="C10" s="5"/>
     </row>
-    <row r="11" spans="2:3" ht="22.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:3" ht="22.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="4" t="s">
         <v>36</v>
       </c>
       <c r="C11" s="5"/>
     </row>
-    <row r="12" spans="2:3" ht="22.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:3" ht="22.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="4" t="s">
         <v>37</v>
       </c>
       <c r="C12" s="5"/>
     </row>
-    <row r="13" spans="2:3" ht="22.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:3" ht="22.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="4" t="s">
         <v>38</v>
       </c>
       <c r="C13" s="5"/>
     </row>
-    <row r="14" spans="2:3" ht="22.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:3" ht="22.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="4" t="s">
         <v>39</v>
       </c>
       <c r="C14" s="5"/>
     </row>
-    <row r="15" spans="2:3" ht="22.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:3" ht="22.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="4" t="s">
         <v>40</v>
       </c>
       <c r="C15" s="5"/>
     </row>
-    <row r="16" spans="2:3" ht="22.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:3" ht="22.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="4" t="s">
         <v>41</v>
       </c>
@@ -1546,21 +1493,21 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="B1:F12"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="30.5546875" customWidth="1"/>
-    <col min="2" max="2" width="50.77734375" customWidth="1"/>
-    <col min="3" max="3" width="67.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="23.109375" customWidth="1"/>
-    <col min="5" max="5" width="18.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="41.77734375" customWidth="1"/>
+    <col min="1" max="1" width="30.5703125" customWidth="1"/>
+    <col min="2" max="2" width="50.7109375" customWidth="1"/>
+    <col min="3" max="3" width="67.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23.140625" customWidth="1"/>
+    <col min="5" max="5" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="41.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:6" ht="16.8" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="2:6" ht="18" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:6" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="2:6" ht="18.75" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
         <v>84</v>
       </c>
@@ -1577,7 +1524,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="3" spans="2:6" ht="18" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B3" s="5" t="s">
         <v>9</v>
       </c>
@@ -1590,7 +1537,7 @@
       </c>
       <c r="F3" s="5"/>
     </row>
-    <row r="4" spans="2:6" ht="18" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B4" s="5" t="s">
         <v>10</v>
       </c>
@@ -1603,7 +1550,7 @@
       </c>
       <c r="F4" s="5"/>
     </row>
-    <row r="5" spans="2:6" ht="18" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B5" s="5" t="s">
         <v>11</v>
       </c>
@@ -1614,7 +1561,7 @@
       <c r="E5" s="5"/>
       <c r="F5" s="5"/>
     </row>
-    <row r="6" spans="2:6" ht="18" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B6" s="5" t="s">
         <v>12</v>
       </c>
@@ -1625,7 +1572,7 @@
       <c r="E6" s="5"/>
       <c r="F6" s="5"/>
     </row>
-    <row r="7" spans="2:6" ht="18" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B7" s="5" t="s">
         <v>13</v>
       </c>
@@ -1636,7 +1583,7 @@
       <c r="E7" s="5"/>
       <c r="F7" s="5"/>
     </row>
-    <row r="8" spans="2:6" ht="18" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B8" s="5" t="s">
         <v>14</v>
       </c>
@@ -1647,7 +1594,7 @@
       <c r="E8" s="5"/>
       <c r="F8" s="5"/>
     </row>
-    <row r="9" spans="2:6" ht="18" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B9" s="5" t="s">
         <v>15</v>
       </c>
@@ -1658,7 +1605,7 @@
       <c r="E9" s="5"/>
       <c r="F9" s="5"/>
     </row>
-    <row r="10" spans="2:6" ht="18" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B10" s="5" t="s">
         <v>16</v>
       </c>
@@ -1669,7 +1616,7 @@
       <c r="E10" s="5"/>
       <c r="F10" s="5"/>
     </row>
-    <row r="11" spans="2:6" ht="18" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B11" s="5" t="s">
         <v>17</v>
       </c>
@@ -1680,7 +1627,7 @@
       <c r="E11" s="5"/>
       <c r="F11" s="5"/>
     </row>
-    <row r="12" spans="2:6" ht="18" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B12" s="5" t="s">
         <v>18</v>
       </c>
@@ -1741,12 +1688,12 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95389844-5F5C-45D5-A5EC-28DEC01E6666}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>89</v>
       </c>
@@ -1754,7 +1701,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>91</v>
       </c>
@@ -1762,7 +1709,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C3" t="s">
         <v>102</v>
       </c>
@@ -1772,17 +1719,17 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="B2:F8"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="31" customWidth="1"/>
-    <col min="2" max="2" width="30.21875" customWidth="1"/>
-    <col min="3" max="6" width="25.109375" customWidth="1"/>
+    <col min="2" max="2" width="30.28515625" customWidth="1"/>
+    <col min="3" max="6" width="25.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:6" ht="18" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:6" ht="18.75" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
         <v>42</v>
       </c>
@@ -1799,7 +1746,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="3" spans="2:6" ht="18" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B3" s="5" t="s">
         <v>47</v>
       </c>
@@ -1808,7 +1755,7 @@
       <c r="E3" s="5"/>
       <c r="F3" s="5"/>
     </row>
-    <row r="4" spans="2:6" ht="18" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B4" s="5" t="s">
         <v>48</v>
       </c>
@@ -1817,7 +1764,7 @@
       <c r="E4" s="5"/>
       <c r="F4" s="5"/>
     </row>
-    <row r="5" spans="2:6" ht="18" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B5" s="5" t="s">
         <v>49</v>
       </c>
@@ -1826,7 +1773,7 @@
       <c r="E5" s="5"/>
       <c r="F5" s="5"/>
     </row>
-    <row r="6" spans="2:6" ht="18" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B6" s="5" t="s">
         <v>50</v>
       </c>
@@ -1835,7 +1782,7 @@
       <c r="E6" s="5"/>
       <c r="F6" s="5"/>
     </row>
-    <row r="7" spans="2:6" ht="18" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B7" s="5" t="s">
         <v>51</v>
       </c>
@@ -1844,7 +1791,7 @@
       <c r="E7" s="5"/>
       <c r="F7" s="5"/>
     </row>
-    <row r="8" spans="2:6" ht="18" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B8" s="5" t="s">
         <v>52</v>
       </c>
@@ -1859,18 +1806,18 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="B1:F8"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="30.33203125" customWidth="1"/>
-    <col min="2" max="2" width="29.33203125" customWidth="1"/>
-    <col min="3" max="6" width="21.6640625" customWidth="1"/>
+    <col min="1" max="1" width="30.28515625" customWidth="1"/>
+    <col min="2" max="2" width="29.28515625" customWidth="1"/>
+    <col min="3" max="6" width="21.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:6" ht="16.8" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="2:6" ht="18" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:6" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="2:6" ht="18.75" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
         <v>42</v>
       </c>
@@ -1887,7 +1834,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="3" spans="2:6" ht="18" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B3" s="5" t="s">
         <v>47</v>
       </c>
@@ -1904,7 +1851,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="4" spans="2:6" ht="18" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B4" s="5" t="s">
         <v>48</v>
       </c>
@@ -1921,7 +1868,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="5" spans="2:6" ht="18" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B5" s="5" t="s">
         <v>49</v>
       </c>
@@ -1938,7 +1885,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="6" spans="2:6" ht="18" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B6" s="5" t="s">
         <v>50</v>
       </c>
@@ -1955,7 +1902,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="7" spans="2:6" ht="18" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B7" s="5" t="s">
         <v>51</v>
       </c>
@@ -1972,7 +1919,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="8" spans="2:6" ht="18" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B8" s="5" t="s">
         <v>52</v>
       </c>
@@ -1995,18 +1942,18 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="B1:C14"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="30.21875" customWidth="1"/>
-    <col min="2" max="2" width="30.6640625" customWidth="1"/>
-    <col min="3" max="3" width="78.6640625" customWidth="1"/>
+    <col min="1" max="1" width="30.28515625" customWidth="1"/>
+    <col min="2" max="2" width="30.7109375" customWidth="1"/>
+    <col min="3" max="3" width="78.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:3" ht="16.8" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="2:3" ht="18" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:3" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="2:3" ht="18.75" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
         <v>28</v>
       </c>
@@ -2014,73 +1961,73 @@
         <v>64</v>
       </c>
     </row>
-    <row r="3" spans="2:3" ht="18" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B3" s="5" t="s">
         <v>65</v>
       </c>
       <c r="C3" s="5"/>
     </row>
-    <row r="4" spans="2:3" ht="18" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B4" s="5" t="s">
         <v>66</v>
       </c>
       <c r="C4" s="5"/>
     </row>
-    <row r="5" spans="2:3" ht="18" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B5" s="5" t="s">
         <v>67</v>
       </c>
       <c r="C5" s="5"/>
     </row>
-    <row r="6" spans="2:3" ht="18" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B6" s="5" t="s">
         <v>68</v>
       </c>
       <c r="C6" s="5"/>
     </row>
-    <row r="7" spans="2:3" ht="18" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B7" s="5" t="s">
         <v>69</v>
       </c>
       <c r="C7" s="5"/>
     </row>
-    <row r="8" spans="2:3" ht="18" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B8" s="5" t="s">
         <v>70</v>
       </c>
       <c r="C8" s="5"/>
     </row>
-    <row r="9" spans="2:3" ht="18" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B9" s="5" t="s">
         <v>71</v>
       </c>
       <c r="C9" s="5"/>
     </row>
-    <row r="10" spans="2:3" ht="18" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B10" s="5" t="s">
         <v>72</v>
       </c>
       <c r="C10" s="5"/>
     </row>
-    <row r="11" spans="2:3" ht="18" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B11" s="5" t="s">
         <v>7</v>
       </c>
       <c r="C11" s="5"/>
     </row>
-    <row r="12" spans="2:3" ht="18" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B12" s="5" t="s">
         <v>73</v>
       </c>
       <c r="C12" s="5"/>
     </row>
-    <row r="13" spans="2:3" ht="18" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B13" s="5" t="s">
         <v>74</v>
       </c>
       <c r="C13" s="5"/>
     </row>
-    <row r="14" spans="2:3" ht="18" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B14" s="5" t="s">
         <v>8</v>
       </c>
@@ -2092,18 +2039,18 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="B2:F10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="30.5546875" customWidth="1"/>
+    <col min="1" max="1" width="30.5703125" customWidth="1"/>
     <col min="2" max="5" width="29" customWidth="1"/>
-    <col min="6" max="6" width="46.77734375" customWidth="1"/>
+    <col min="6" max="6" width="46.7109375" customWidth="1"/>
     <col min="7" max="7" width="29" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:6" ht="18" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:6" ht="18.75" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
         <v>75</v>
       </c>
@@ -2120,7 +2067,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="3" spans="2:6" ht="18" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B3" s="5" t="s">
         <v>92</v>
       </c>
@@ -2131,7 +2078,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="4" spans="2:6" ht="18" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B4" s="5" t="s">
         <v>93</v>
       </c>
@@ -2142,7 +2089,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="5" spans="2:6" ht="18" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B5" s="5" t="s">
         <v>94</v>
       </c>
@@ -2153,7 +2100,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="6" spans="2:6" ht="18" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B6" s="5" t="s">
         <v>95</v>
       </c>
@@ -2162,7 +2109,7 @@
       <c r="E6" s="5"/>
       <c r="F6" s="6"/>
     </row>
-    <row r="7" spans="2:6" ht="18" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B7" s="5" t="s">
         <v>96</v>
       </c>
@@ -2171,7 +2118,7 @@
       <c r="E7" s="5"/>
       <c r="F7" s="6"/>
     </row>
-    <row r="8" spans="2:6" ht="18" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B8" s="5" t="s">
         <v>97</v>
       </c>
@@ -2180,7 +2127,7 @@
       <c r="E8" s="5"/>
       <c r="F8" s="6"/>
     </row>
-    <row r="9" spans="2:6" ht="18" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B9" s="5" t="s">
         <v>98</v>
       </c>
@@ -2189,7 +2136,7 @@
       <c r="E9" s="5"/>
       <c r="F9" s="6"/>
     </row>
-    <row r="10" spans="2:6" ht="18" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B10" s="5" t="s">
         <v>99</v>
       </c>
@@ -2269,17 +2216,17 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B7EF1668-A45A-4B23-A7DB-2952BC350BA3}">
   <dimension ref="B2:C12"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="34.5546875" customWidth="1"/>
-    <col min="2" max="2" width="43.44140625" customWidth="1"/>
-    <col min="3" max="3" width="108.44140625" customWidth="1"/>
+    <col min="1" max="1" width="34.5703125" customWidth="1"/>
+    <col min="2" max="2" width="43.42578125" customWidth="1"/>
+    <col min="3" max="3" width="108.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:3" ht="18" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:3" ht="18.75" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
         <v>112</v>
       </c>
@@ -2287,7 +2234,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="3" spans="2:3" ht="22.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:3" ht="22.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="4" t="s">
         <v>107</v>
       </c>
@@ -2295,7 +2242,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="4" spans="2:3" ht="22.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:3" ht="22.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="4" t="s">
         <v>108</v>
       </c>
@@ -2303,7 +2250,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="5" spans="2:3" ht="22.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:3" ht="22.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="4" t="s">
         <v>109</v>
       </c>
@@ -2311,7 +2258,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="6" spans="2:3" ht="22.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:3" ht="22.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="4" t="s">
         <v>110</v>
       </c>
@@ -2319,7 +2266,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="7" spans="2:3" ht="22.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:3" ht="22.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="4" t="s">
         <v>121</v>
       </c>
@@ -2327,7 +2274,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="8" spans="2:3" ht="22.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:3" ht="22.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="4" t="s">
         <v>111</v>
       </c>
@@ -2335,7 +2282,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="9" spans="2:3" ht="22.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:3" ht="22.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="4" t="s">
         <v>76</v>
       </c>
@@ -2343,7 +2290,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="10" spans="2:3" ht="22.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:3" ht="22.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="4" t="s">
         <v>114</v>
       </c>
@@ -2351,7 +2298,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="11" spans="2:3" ht="22.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:3" ht="22.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="4" t="s">
         <v>115</v>
       </c>
@@ -2359,7 +2306,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="12" spans="2:3" ht="22.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:3" ht="22.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="4" t="s">
         <v>116</v>
       </c>

</xml_diff>

<commit_message>
Kit gratis (Excel): logo -> solo el isotipo MM (cuadrado), sin wordmark
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/landing/assets/Menttor_Kit_Inicio_Rapido.xlsx
+++ b/landing/assets/Menttor_Kit_Inicio_Rapido.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JOSEMO~1\AppData\Local\Temp\claude\C--Users-Jose-Montilla-OneDrive-Cloude-pagina-web-MM\82739746-f994-4b96-ab4e-13fcee2a012b\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA0460D5-B49B-4573-8F08-5C555BB9227C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86DDD9B6-B308-4DE8-9C5C-BA62E13C7B8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="808" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -587,16 +587,16 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>2072640</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>222780</xdr:rowOff>
+      <xdr:colOff>685800</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Imagen 3">
+        <xdr:cNvPr id="3" name="Imagen 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0B36EA55-F646-850D-D599-6A52FEAFD52E}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8F742D4E-1377-4C30-042F-A62EAA04EEB2}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -619,7 +619,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="2072640" cy="651405"/>
+          <a:ext cx="685800" cy="685800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -642,16 +642,16 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>2072640</xdr:colOff>
+      <xdr:colOff>685800</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>222780</xdr:rowOff>
+      <xdr:rowOff>257175</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Imagen 3">
+        <xdr:cNvPr id="3" name="Imagen 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4DD91091-5757-10EC-41C5-7BA5669C8B17}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4F5B46CC-0636-7DCA-0165-05FB1E2A5C24}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -674,7 +674,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="2072640" cy="651405"/>
+          <a:ext cx="685800" cy="685800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -697,16 +697,16 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>2034540</xdr:colOff>
+      <xdr:colOff>685800</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>184347</xdr:rowOff>
+      <xdr:rowOff>230717</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Imagen 3">
+        <xdr:cNvPr id="3" name="Imagen 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DCA4B3D6-AC33-723C-98FD-1B6D3CFBFFD3}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{750AF3F6-7452-CBB8-8277-36290D60589D}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -729,7 +729,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="2034540" cy="639430"/>
+          <a:ext cx="685800" cy="685800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -752,16 +752,16 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>2063115</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>219786</xdr:rowOff>
+      <xdr:colOff>685800</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Imagen 3">
+        <xdr:cNvPr id="3" name="Imagen 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D33DA621-7111-13D5-1368-73C2C1845BCE}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0FA23912-7E72-7BCA-4C9C-C78FE59D1ABA}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -784,7 +784,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="2063115" cy="648411"/>
+          <a:ext cx="685800" cy="685800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -807,16 +807,16 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>2015490</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>185768</xdr:rowOff>
+      <xdr:colOff>685800</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Imagen 3">
+        <xdr:cNvPr id="3" name="Imagen 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D82E59FB-E6BF-351D-6AC3-2AED3B60777B}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0E772637-B701-A604-E6AE-5CB87485F1DC}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -839,7 +839,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="2015490" cy="633443"/>
+          <a:ext cx="685800" cy="685800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -861,17 +861,17 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>186966</xdr:rowOff>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>685800</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Imagen 3">
+        <xdr:cNvPr id="3" name="Imagen 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9374BFF1-C3BC-5BF8-E72D-65C556BF927B}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DD98ACCF-A55B-94EE-1F08-A768066D406D}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -894,7 +894,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="2019300" cy="634641"/>
+          <a:ext cx="685800" cy="685800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -917,16 +917,16 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>2034540</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>210805</xdr:rowOff>
+      <xdr:colOff>685800</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Imagen 3">
+        <xdr:cNvPr id="3" name="Imagen 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6BF38672-04AB-2C08-71B1-2694968A08E1}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7AD4B9C7-A70A-A98B-D50A-DA561599762A}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -949,7 +949,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="2034540" cy="639430"/>
+          <a:ext cx="685800" cy="685800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -972,16 +972,16 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>2072640</xdr:colOff>
+      <xdr:colOff>685800</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>222780</xdr:rowOff>
+      <xdr:rowOff>257175</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Imagen 3">
+        <xdr:cNvPr id="3" name="Imagen 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F730F1E2-3DF5-7BE4-CE4A-E67123706F00}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A0AC8440-91D5-A1F3-739E-512983B7C9FD}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1004,7 +1004,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="2072640" cy="651405"/>
+          <a:ext cx="685800" cy="685800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>

</xml_diff>

<commit_message>
Kit Excel gratis: agrandar isotipo MM (54pt -> 130pt) en las 8 hojas
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/landing/assets/Menttor_Kit_Inicio_Rapido.xlsx
+++ b/landing/assets/Menttor_Kit_Inicio_Rapido.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JOSEMO~1\AppData\Local\Temp\claude\C--Users-Jose-Montilla-OneDrive-Cloude-pagina-web-MM\82739746-f994-4b96-ab4e-13fcee2a012b\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86DDD9B6-B308-4DE8-9C5C-BA62E13C7B8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0A46B29-38E2-48F8-AD4C-F6ED5E1E4B77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="808" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -587,16 +587,16 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>685800</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
+      <xdr:colOff>1651000</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>31750</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Imagen 2">
+        <xdr:cNvPr id="4" name="Imagen 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8F742D4E-1377-4C30-042F-A62EAA04EEB2}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8BB67733-2BD6-F788-5486-A05533710C22}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -619,7 +619,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="685800" cy="685800"/>
+          <a:ext cx="1651000" cy="1651000"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -642,16 +642,16 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>685800</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>257175</xdr:rowOff>
+      <xdr:colOff>1651000</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>117475</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Imagen 2">
+        <xdr:cNvPr id="4" name="Imagen 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4F5B46CC-0636-7DCA-0165-05FB1E2A5C24}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EA2368C8-D2BC-C594-A00B-A85DE47873AA}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -674,7 +674,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="685800" cy="685800"/>
+          <a:ext cx="1651000" cy="1651000"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -697,16 +697,16 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>685800</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>230717</xdr:rowOff>
+      <xdr:colOff>1651000</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>222250</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Imagen 2">
+        <xdr:cNvPr id="4" name="Imagen 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{750AF3F6-7452-CBB8-8277-36290D60589D}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CC569837-DC1B-BDD5-20F0-523A40EE3A0A}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -729,7 +729,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="685800" cy="685800"/>
+          <a:ext cx="1651000" cy="1651000"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -752,16 +752,16 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>685800</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
+      <xdr:colOff>1651000</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>31750</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Imagen 2">
+        <xdr:cNvPr id="4" name="Imagen 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0FA23912-7E72-7BCA-4C9C-C78FE59D1ABA}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EA88E7FC-4487-90B8-ED1C-560CF84E1695}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -784,7 +784,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="685800" cy="685800"/>
+          <a:ext cx="1651000" cy="1651000"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -807,16 +807,16 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>685800</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:colOff>1651000</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>12700</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Imagen 2">
+        <xdr:cNvPr id="4" name="Imagen 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0E772637-B701-A604-E6AE-5CB87485F1DC}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A97D2932-5E7B-EE88-EBBD-24D0015B86A2}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -839,7 +839,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="685800" cy="685800"/>
+          <a:ext cx="1651000" cy="1651000"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -862,16 +862,16 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>685800</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:colOff>1651000</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>12700</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Imagen 2">
+        <xdr:cNvPr id="4" name="Imagen 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DD98ACCF-A55B-94EE-1F08-A768066D406D}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{588D88D7-2373-A14B-6170-90FA5D50E7C6}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -894,7 +894,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="685800" cy="685800"/>
+          <a:ext cx="1651000" cy="1651000"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -917,16 +917,16 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>685800</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
+      <xdr:colOff>1651000</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>31750</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Imagen 2">
+        <xdr:cNvPr id="4" name="Imagen 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7AD4B9C7-A70A-A98B-D50A-DA561599762A}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{248906B7-AABE-7C7C-6AD5-CE71049856D4}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -949,7 +949,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="685800" cy="685800"/>
+          <a:ext cx="1651000" cy="1651000"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -972,16 +972,16 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>685800</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>257175</xdr:rowOff>
+      <xdr:colOff>1651000</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>117475</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Imagen 2">
+        <xdr:cNvPr id="4" name="Imagen 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A0AC8440-91D5-A1F3-739E-512983B7C9FD}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E10F5C4A-78C4-D264-047A-C13E693795EE}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1004,7 +1004,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="685800" cy="685800"/>
+          <a:ext cx="1651000" cy="1651000"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>

</xml_diff>